<commit_message>
Rebuild the BRD-13 migration pack without migration wave codes and internal source names
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-13_Data_Migration/BIBS_Migration_BRD-13_Cutover_Task_Plan_v1.2.xlsx
+++ b/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-13_Data_Migration/BIBS_Migration_BRD-13_Cutover_Task_Plan_v1.2.xlsx
@@ -2038,7 +2038,7 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>No open Critical or High defect; Medium defects have an agreed fix date</t>
+          <t>No open Critical or High issue; Medium issues have an agreed fix date</t>
         </is>
       </c>
       <c r="C5" s="12" t="n"/>
@@ -4593,7 +4593,7 @@
       <c r="D9" s="12" t="inlineStr"/>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Production environment ready - BIBS release of the go-live build deployed, MIG_ENVIRONMENT_CLASS = PRODUCTION, MIG_CUTOVER_DATE = T, MIG_OPENING_VALUE_DATE = 1-Jan-2028, MIG_GOLIVE_RENEWAL_TO = 31-May-2028, MIG_RENEWAL_URGENT_TO = 31-Jan-2028, jobs scheduled</t>
+          <t>Production environment ready - BIBS release of the go-live release deployed, MIG_ENVIRONMENT_CLASS = PRODUCTION, MIG_CUTOVER_DATE = T, MIG_OPENING_VALUE_DATE = 1-Jan-2028, MIG_GOLIVE_RENEWAL_TO = 31-May-2028, MIG_RENEWAL_URGENT_TO = 31-Jan-2028, jobs scheduled</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E62" s="12" t="inlineStr">
         <is>
-          <t>Prepare the go / no-go pack - MIG-GONOGO with measured criteria, open defects, sign-off status</t>
+          <t>Prepare the go / no-go pack - MIG-GONOGO with measured criteria, open issues, sign-off status</t>
         </is>
       </c>
       <c r="F62" s="12" t="inlineStr">
@@ -7903,7 +7903,7 @@
       </c>
       <c r="E72" s="12" t="inlineStr">
         <is>
-          <t>Midday check - defects, queues, Migration Clearing still 0.00, no legacy business posting</t>
+          <t>Midday check - issues, queues, Migration Clearing still 0.00, no legacy business posting</t>
         </is>
       </c>
       <c r="F72" s="12" t="inlineStr">
@@ -8115,7 +8115,7 @@
       <c r="D76" s="12" t="inlineStr"/>
       <c r="E76" s="12" t="inlineStr">
         <is>
-          <t>Defect triage twice a day (10:00 and 16:00) with Operations, Comptrollership, Renewal and iorta QA</t>
+          <t>Issue triage twice a day (10:00 and 16:00) with Operations, Comptrollership, Renewal and iorta QA</t>
         </is>
       </c>
       <c r="F76" s="12" t="inlineStr">
@@ -8133,7 +8133,7 @@
       </c>
       <c r="I76" s="12" t="inlineStr">
         <is>
-          <t>Defect log updated; severity agreed</t>
+          <t>Issue log updated; severity agreed</t>
         </is>
       </c>
       <c r="J76" s="12" t="inlineStr"/>
@@ -8315,7 +8315,7 @@
       <c r="D80" s="12" t="inlineStr"/>
       <c r="E80" s="12" t="inlineStr">
         <is>
-          <t>Week-1 review with the board - defects, volumes, performance, renewal queue, user feedback</t>
+          <t>Week-1 review with the board - issues, volumes, performance, renewal queue, user feedback</t>
         </is>
       </c>
       <c r="F80" s="12" t="inlineStr">
@@ -9686,7 +9686,7 @@
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t>iorta TechNXT QA (smoke tests, defect triage)</t>
+          <t>iorta TechNXT QA (smoke tests, issue triage)</t>
         </is>
       </c>
       <c r="C20" s="12" t="inlineStr">
@@ -10734,7 +10734,7 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>No open Critical defect of the migration or of a Day-1 module</t>
+          <t>No open Critical issue of the migration or of a Day-1 module</t>
         </is>
       </c>
       <c r="F12" s="12" t="n"/>
@@ -11301,7 +11301,7 @@
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>No Critical defect that stops receipts, payment application, remittance or booking</t>
+          <t>No Critical issue that stops receipts, payment application, remittance or booking</t>
         </is>
       </c>
       <c r="F33" s="12" t="n"/>
@@ -11720,7 +11720,7 @@
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>Hotfix of a Critical defect approved by the go / no-go board</t>
+          <t>Hotfix of a Critical issue approved by the go / no-go board</t>
         </is>
       </c>
     </row>

</xml_diff>